<commit_message>
fim with tariffs + uncertainty
</commit_message>
<xml_diff>
--- a/results/04-2025/beta/contributions-04-2025.xlsx
+++ b/results/04-2025/beta/contributions-04-2025.xlsx
@@ -22334,13 +22334,13 @@
         <v>-0.102182602654285</v>
       </c>
       <c r="AC223" t="n">
-        <v>0.0391316499056623</v>
+        <v>-0.960868350094338</v>
       </c>
       <c r="AD223" t="n">
-        <v>-0.409229395446914</v>
+        <v>-1.40922939544691</v>
       </c>
       <c r="AE223" t="n">
-        <v>-0.037698433586331</v>
+        <v>-0.287698433586331</v>
       </c>
     </row>
     <row r="224">
@@ -22429,13 +22429,13 @@
         <v>0.0369005845804345</v>
       </c>
       <c r="AC224" t="n">
-        <v>0.199220473680243</v>
+        <v>-0.800779526319757</v>
       </c>
       <c r="AD224" t="n">
-        <v>-0.155248931431897</v>
+        <v>-1.1552489314319</v>
       </c>
       <c r="AE224" t="n">
-        <v>-0.201868678957015</v>
+        <v>-0.701868678957015</v>
       </c>
     </row>
     <row r="225">
@@ -22524,13 +22524,13 @@
         <v>0.0318501921225512</v>
       </c>
       <c r="AC225" t="n">
-        <v>0.0975348743533302</v>
+        <v>-0.90246512564667</v>
       </c>
       <c r="AD225" t="n">
-        <v>-0.253775898254652</v>
+        <v>-1.25377589825465</v>
       </c>
       <c r="AE225" t="n">
-        <v>-0.361140330962118</v>
+        <v>-1.11114033096212</v>
       </c>
     </row>
     <row r="226">
@@ -22619,13 +22619,13 @@
         <v>-0.08004016235873</v>
       </c>
       <c r="AC226" t="n">
-        <v>0.198973945998221</v>
+        <v>-0.801026054001779</v>
       </c>
       <c r="AD226" t="n">
-        <v>-0.133241235325917</v>
+        <v>-1.13324123532592</v>
       </c>
       <c r="AE226" t="n">
-        <v>-0.237873865114846</v>
+        <v>-1.23787386511485</v>
       </c>
     </row>
     <row r="227">
@@ -22720,7 +22720,7 @@
         <v>-0.187245844022027</v>
       </c>
       <c r="AE227" t="n">
-        <v>-0.182377977258624</v>
+        <v>-0.932377977258624</v>
       </c>
     </row>
     <row r="228">
@@ -22815,7 +22815,7 @@
         <v>-0.262807787422518</v>
       </c>
       <c r="AE228" t="n">
-        <v>-0.209267691256279</v>
+        <v>-0.70926769125628</v>
       </c>
     </row>
     <row r="229">
@@ -22910,7 +22910,7 @@
         <v>-0.318001914660002</v>
       </c>
       <c r="AE229" t="n">
-        <v>-0.225324195357617</v>
+        <v>-0.475324195357617</v>
       </c>
     </row>
     <row r="230">
@@ -23005,7 +23005,7 @@
         <v>-0.609590844482197</v>
       </c>
       <c r="AE230" t="n">
-        <v>-0.344411597646686</v>
+        <v>-0.344411597646687</v>
       </c>
     </row>
     <row r="231">
@@ -23480,7 +23480,7 @@
         <v>0</v>
       </c>
       <c r="AE235" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="236">
@@ -23575,7 +23575,7 @@
         <v>0</v>
       </c>
       <c r="AE236" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="237">
@@ -23670,7 +23670,7 @@
         <v>0</v>
       </c>
       <c r="AE237" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="238">
@@ -23765,7 +23765,7 @@
         <v>0</v>
       </c>
       <c r="AE238" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="239">
@@ -23860,7 +23860,7 @@
         <v>0</v>
       </c>
       <c r="AE239" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="240">
@@ -23955,7 +23955,7 @@
         <v>0</v>
       </c>
       <c r="AE240" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="241">
@@ -24050,7 +24050,7 @@
         <v>0</v>
       </c>
       <c r="AE241" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="242">
@@ -24145,7 +24145,7 @@
         <v>0</v>
       </c>
       <c r="AE242" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="243">
@@ -24240,7 +24240,7 @@
         <v>0</v>
       </c>
       <c r="AE243" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="244">
@@ -24335,7 +24335,7 @@
         <v>0</v>
       </c>
       <c r="AE244" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="245">
@@ -24430,7 +24430,7 @@
         <v>0</v>
       </c>
       <c r="AE245" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="246">
@@ -24525,7 +24525,7 @@
         <v>0</v>
       </c>
       <c r="AE246" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="247">
@@ -24620,7 +24620,7 @@
         <v>0</v>
       </c>
       <c r="AE247" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="248">
@@ -24715,7 +24715,7 @@
         <v>0</v>
       </c>
       <c r="AE248" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="249">
@@ -24810,7 +24810,7 @@
         <v>0</v>
       </c>
       <c r="AE249" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="250">
@@ -24905,7 +24905,7 @@
         <v>0</v>
       </c>
       <c r="AE250" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="251">
@@ -25000,7 +25000,7 @@
         <v>0</v>
       </c>
       <c r="AE251" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="252">
@@ -25095,7 +25095,7 @@
         <v>0</v>
       </c>
       <c r="AE252" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="253">
@@ -25190,7 +25190,7 @@
         <v>0</v>
       </c>
       <c r="AE253" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="254">
@@ -25285,7 +25285,7 @@
         <v>0</v>
       </c>
       <c r="AE254" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="255">
@@ -25380,7 +25380,7 @@
         <v>0</v>
       </c>
       <c r="AE255" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="256">
@@ -25475,7 +25475,7 @@
         <v>0</v>
       </c>
       <c r="AE256" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="257">
@@ -25570,7 +25570,7 @@
         <v>0</v>
       </c>
       <c r="AE257" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="258">
@@ -25665,7 +25665,7 @@
         <v>0</v>
       </c>
       <c r="AE258" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="259">
@@ -25760,7 +25760,7 @@
         <v>0</v>
       </c>
       <c r="AE259" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
     <row r="260">
@@ -25855,7 +25855,7 @@
         <v>0</v>
       </c>
       <c r="AE260" t="n">
-        <v>-0.000000000000000888178419700125</v>
+        <v>-0.00000000000000177635683940025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>